<commit_message>
Se completa [TC-002] Registro fallido por email duplicado
</commit_message>
<xml_diff>
--- a/testData/TutorialsNinja_RegisterPage.xlsx
+++ b/testData/TutorialsNinja_RegisterPage.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/erickfloresovando/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1EF766C-6905-1340-B754-7F5C88F1E5F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38FBCD51-B018-E046-AD62-6460FFECBE43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19200" xr2:uid="{A4E39AE2-BE39-2E44-9441-96961B052630}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15600" xr2:uid="{A4E39AE2-BE39-2E44-9441-96961B052630}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -549,27 +549,27 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D2" s="6">
-        <v>5559876543</v>
+        <v>5551234567</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1" xr:uid="{EFA6B181-151C-3042-85DD-AA36DD5D9A93}"/>
+    <hyperlink ref="C2" r:id="rId1" xr:uid="{5C5E8BDF-807F-974A-926D-5FE93B49A08D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -627,24 +627,24 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A4" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D4" s="6">
-        <v>5551234567</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>23</v>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3" s="6">
+        <v>5559876543</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -690,9 +690,9 @@
   </sheetData>
   <hyperlinks>
     <hyperlink ref="C2" r:id="rId1" xr:uid="{2994E8E3-27A4-3342-A375-5CF20C5E6751}"/>
-    <hyperlink ref="C4" r:id="rId2" xr:uid="{5C5E8BDF-807F-974A-926D-5FE93B49A08D}"/>
-    <hyperlink ref="C5" r:id="rId3" xr:uid="{2ED25ACD-8A16-DD42-8FB2-9069856DDED4}"/>
-    <hyperlink ref="C6" r:id="rId4" xr:uid="{432655B1-7C28-0E40-9862-B8308F8A8DD8}"/>
+    <hyperlink ref="C5" r:id="rId2" xr:uid="{2ED25ACD-8A16-DD42-8FB2-9069856DDED4}"/>
+    <hyperlink ref="C6" r:id="rId3" xr:uid="{432655B1-7C28-0E40-9862-B8308F8A8DD8}"/>
+    <hyperlink ref="C3" r:id="rId4" xr:uid="{A65943FD-A8AA-0141-8300-C953B43F032A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>